<commit_message>
Spreadsheet sample: reconcile to raw export, flag conflicts/typos, live whole-column summary; disclose AI processing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sheets/sample-after.xlsx
+++ b/sheets/sample-after.xlsx
@@ -11,7 +11,8 @@
     <sheet name="Invoices" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Summary" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Duplicates removed" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Checks" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Needs review" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Checks" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -20,10 +21,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
     <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="166" formatCode="&quot;$&quot;#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="mmm yyyy"/>
   </numFmts>
   <fonts count="2">
     <font>
@@ -62,13 +64,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -146,16 +150,15 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Invoices" displayName="Invoices" ref="A1:G61" headerRowCount="1">
-  <autoFilter ref="A1:G61"/>
-  <tableColumns count="7">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="Invoices" displayName="Invoices" ref="A1:F61" headerRowCount="1">
+  <autoFilter ref="A1:F61"/>
+  <tableColumns count="6">
     <tableColumn id="1" name="Invoice"/>
     <tableColumn id="2" name="Date"/>
     <tableColumn id="3" name="Customer"/>
     <tableColumn id="4" name="Service"/>
     <tableColumn id="5" name="Amount"/>
     <tableColumn id="6" name="Status"/>
-    <tableColumn id="7" name="Month"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -450,10 +453,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A6"/>
+  <dimension ref="A1:A7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="110" customWidth="1" min="1" max="1"/>
+    <col width="130" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -469,28 +472,35 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Raw export: 66 rows. Blank rows removed: 1. Duplicate invoices removed: 5.</t>
+          <t>Original export: 67 rows, $88,063.50 in total. Blank rows: 1. Exact duplicates removed: 5. Conflicting re-issues held for review: 1. Possible name typos flagged: 1.</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Fixed: 4 date formats -&gt; real dates; amounts stored as text ($, commas, 'AUD') -&gt; numbers;</t>
+          <t>Fixed: 4 date formats -&gt; real dates; amounts stored as text ($, commas, 'AUD') -&gt; numbers; stray spaces/capitals in names;</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>customer names with stray spaces/capitals merged; Paid? (Y/yes/Paid/blank) -&gt; Paid/Unpaid dropdown.</t>
+          <t>Paid? (Y/yes/Paid, N/no, blank) -&gt; Paid / Unpaid / Unknown dropdown. Blank is Unknown, never assumed Unpaid.</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Summary and Checks sheets are live formulas, so they keep working when new rows are added to the table.</t>
+          <t>Nothing is deleted silently: duplicates and anything ambiguous are on their own sheets with the reason.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Summary uses whole-column formulas: rows you add on Invoices are included. Checks flags a new customer missing from Summary.</t>
         </is>
       </c>
     </row>
@@ -505,7 +515,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G61"/>
+  <dimension ref="A1:F61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -513,8 +523,7 @@
     <col width="22" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="10" customWidth="1" min="7" max="7"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -548,11 +557,6 @@
           <t>Status</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -581,10 +585,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G2">
-        <f>TEXT(B2,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -613,10 +613,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G3">
-        <f>TEXT(B3,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -645,10 +641,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G4">
-        <f>TEXT(B4,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -677,10 +669,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G5">
-        <f>TEXT(B5,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -709,10 +697,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G6">
-        <f>TEXT(B6,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -741,10 +725,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G7">
-        <f>TEXT(B7,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -773,10 +753,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G8">
-        <f>TEXT(B8,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -805,10 +781,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G9">
-        <f>TEXT(B9,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -837,10 +809,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G10">
-        <f>TEXT(B10,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -869,10 +837,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G11">
-        <f>TEXT(B11,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -898,12 +862,8 @@
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G12">
-        <f>TEXT(B12,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="13">
@@ -930,12 +890,8 @@
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G13">
-        <f>TEXT(B13,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="14">
@@ -962,12 +918,8 @@
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G14">
-        <f>TEXT(B14,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="15">
@@ -997,10 +949,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G15">
-        <f>TEXT(B15,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1029,10 +977,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G16">
-        <f>TEXT(B16,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1058,12 +1002,8 @@
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G17">
-        <f>TEXT(B17,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="18">
@@ -1093,10 +1033,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G18">
-        <f>TEXT(B18,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1125,10 +1061,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G19">
-        <f>TEXT(B19,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1157,10 +1089,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G20">
-        <f>TEXT(B20,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1189,10 +1117,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G21">
-        <f>TEXT(B21,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1221,10 +1145,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G22">
-        <f>TEXT(B22,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1253,10 +1173,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G23">
-        <f>TEXT(B23,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1282,12 +1198,8 @@
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G24">
-        <f>TEXT(B24,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="25">
@@ -1317,10 +1229,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G25">
-        <f>TEXT(B25,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1349,10 +1257,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G26">
-        <f>TEXT(B26,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1381,10 +1285,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G27">
-        <f>TEXT(B27,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1413,10 +1313,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G28">
-        <f>TEXT(B28,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1445,10 +1341,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G29">
-        <f>TEXT(B29,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1477,10 +1369,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G30">
-        <f>TEXT(B30,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1509,10 +1397,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G31">
-        <f>TEXT(B31,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1538,12 +1422,8 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G32">
-        <f>TEXT(B32,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="33">
@@ -1573,10 +1453,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G33">
-        <f>TEXT(B33,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1589,7 +1465,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Oakridge Motors</t>
+          <t>Parkside Dentl</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -1605,10 +1481,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G34">
-        <f>TEXT(B34,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1637,10 +1509,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G35">
-        <f>TEXT(B35,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1666,12 +1534,8 @@
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G36">
-        <f>TEXT(B36,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="37">
@@ -1698,12 +1562,8 @@
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G37">
-        <f>TEXT(B37,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="38">
@@ -1733,10 +1593,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G38">
-        <f>TEXT(B38,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1765,10 +1621,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G39">
-        <f>TEXT(B39,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1797,10 +1649,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G40">
-        <f>TEXT(B40,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1826,12 +1674,8 @@
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G41">
-        <f>TEXT(B41,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="42">
@@ -1861,10 +1705,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G42">
-        <f>TEXT(B42,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1890,12 +1730,8 @@
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G43">
-        <f>TEXT(B43,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="44">
@@ -1925,10 +1761,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G44">
-        <f>TEXT(B44,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1957,10 +1789,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G45">
-        <f>TEXT(B45,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -1989,10 +1817,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G46">
-        <f>TEXT(B46,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2021,10 +1845,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G47">
-        <f>TEXT(B47,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2053,10 +1873,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G48">
-        <f>TEXT(B48,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2085,10 +1901,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G49">
-        <f>TEXT(B49,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2117,10 +1929,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G50">
-        <f>TEXT(B50,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2149,10 +1957,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G51">
-        <f>TEXT(B51,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2181,10 +1985,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G52">
-        <f>TEXT(B52,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2213,10 +2013,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G53">
-        <f>TEXT(B53,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2245,10 +2041,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G54">
-        <f>TEXT(B54,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2277,10 +2069,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G55">
-        <f>TEXT(B55,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2309,10 +2097,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G56">
-        <f>TEXT(B56,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2338,12 +2122,8 @@
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Unpaid</t>
-        </is>
-      </c>
-      <c r="G57">
-        <f>TEXT(B57,"yyyy-mm")</f>
-        <v/>
+          <t>Unknown</t>
+        </is>
       </c>
     </row>
     <row r="58">
@@ -2373,10 +2153,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G58">
-        <f>TEXT(B58,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2405,10 +2181,6 @@
           <t>Unpaid</t>
         </is>
       </c>
-      <c r="G59">
-        <f>TEXT(B59,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2437,10 +2209,6 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G60">
-        <f>TEXT(B60,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2469,15 +2237,11 @@
           <t>Paid</t>
         </is>
       </c>
-      <c r="G61">
-        <f>TEXT(B61,"yyyy-mm")</f>
-        <v/>
-      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="F2:F261" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
-      <formula1>"Paid,Unpaid"</formula1>
+    <dataValidation sqref="F2:F561" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="0" type="list">
+      <formula1>"Paid,Unpaid,Unknown"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2493,19 +2257,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D17"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
-    <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="14" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Summary (live formulas: edit the Invoices sheet and these update)</t>
+          <t>Summary (live: add or edit rows on Invoices and this updates; new customers need a row here, and Checks flags it)</t>
         </is>
       </c>
     </row>
@@ -2527,6 +2292,11 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
+          <t>Status unknown</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
           <t>Jobs</t>
         </is>
       </c>
@@ -2538,15 +2308,19 @@
         </is>
       </c>
       <c r="B4" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A4)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A4)</f>
         <v/>
       </c>
       <c r="C4" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A4,Invoices!$F$2:$F$61,"Unpaid")</f>
-        <v/>
-      </c>
-      <c r="D4">
-        <f>COUNTIF(Invoices!$C$2:$C$61,A4)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A4,Invoices!$F:$F,"Unpaid")</f>
+        <v/>
+      </c>
+      <c r="D4" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A4,Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="E4">
+        <f>COUNTIF(Invoices!$C:$C,A4)</f>
         <v/>
       </c>
     </row>
@@ -2557,15 +2331,19 @@
         </is>
       </c>
       <c r="B5" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A5)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A5)</f>
         <v/>
       </c>
       <c r="C5" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A5,Invoices!$F$2:$F$61,"Unpaid")</f>
-        <v/>
-      </c>
-      <c r="D5">
-        <f>COUNTIF(Invoices!$C$2:$C$61,A5)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A5,Invoices!$F:$F,"Unpaid")</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A5,Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="E5">
+        <f>COUNTIF(Invoices!$C:$C,A5)</f>
         <v/>
       </c>
     </row>
@@ -2576,15 +2354,19 @@
         </is>
       </c>
       <c r="B6" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A6)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A6)</f>
         <v/>
       </c>
       <c r="C6" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A6,Invoices!$F$2:$F$61,"Unpaid")</f>
-        <v/>
-      </c>
-      <c r="D6">
-        <f>COUNTIF(Invoices!$C$2:$C$61,A6)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A6,Invoices!$F:$F,"Unpaid")</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A6,Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="E6">
+        <f>COUNTIF(Invoices!$C:$C,A6)</f>
         <v/>
       </c>
     </row>
@@ -2595,15 +2377,19 @@
         </is>
       </c>
       <c r="B7" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A7)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A7)</f>
         <v/>
       </c>
       <c r="C7" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A7,Invoices!$F$2:$F$61,"Unpaid")</f>
-        <v/>
-      </c>
-      <c r="D7">
-        <f>COUNTIF(Invoices!$C$2:$C$61,A7)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A7,Invoices!$F:$F,"Unpaid")</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A7,Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="E7">
+        <f>COUNTIF(Invoices!$C:$C,A7)</f>
         <v/>
       </c>
     </row>
@@ -2614,15 +2400,19 @@
         </is>
       </c>
       <c r="B8" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A8)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A8)</f>
         <v/>
       </c>
       <c r="C8" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A8,Invoices!$F$2:$F$61,"Unpaid")</f>
-        <v/>
-      </c>
-      <c r="D8">
-        <f>COUNTIF(Invoices!$C$2:$C$61,A8)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A8,Invoices!$F:$F,"Unpaid")</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A8,Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="E8">
+        <f>COUNTIF(Invoices!$C:$C,A8)</f>
         <v/>
       </c>
     </row>
@@ -2633,127 +2423,264 @@
         </is>
       </c>
       <c r="B9" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A9)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A9)</f>
         <v/>
       </c>
       <c r="C9" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A9,Invoices!$F$2:$F$61,"Unpaid")</f>
-        <v/>
-      </c>
-      <c r="D9">
-        <f>COUNTIF(Invoices!$C$2:$C$61,A9)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A9,Invoices!$F:$F,"Unpaid")</f>
+        <v/>
+      </c>
+      <c r="D9" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A9,Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="E9">
+        <f>COUNTIF(Invoices!$C:$C,A9)</f>
         <v/>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Riverbend Vets</t>
+          <t>Parkside Dentl</t>
         </is>
       </c>
       <c r="B10" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A10)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A10)</f>
         <v/>
       </c>
       <c r="C10" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A10,Invoices!$F$2:$F$61,"Unpaid")</f>
-        <v/>
-      </c>
-      <c r="D10">
-        <f>COUNTIF(Invoices!$C$2:$C$61,A10)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A10,Invoices!$F:$F,"Unpaid")</f>
+        <v/>
+      </c>
+      <c r="D10" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A10,Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="E10">
+        <f>COUNTIF(Invoices!$C:$C,A10)</f>
         <v/>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Summit Physio</t>
+          <t>Riverbend Vets</t>
         </is>
       </c>
       <c r="B11" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A11)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A11)</f>
         <v/>
       </c>
       <c r="C11" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$C$2:$C$61,A11,Invoices!$F$2:$F$61,"Unpaid")</f>
-        <v/>
-      </c>
-      <c r="D11">
-        <f>COUNTIF(Invoices!$C$2:$C$61,A11)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A11,Invoices!$F:$F,"Unpaid")</f>
+        <v/>
+      </c>
+      <c r="D11" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A11,Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="E11">
+        <f>COUNTIF(Invoices!$C:$C,A11)</f>
         <v/>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>Summit Physio</t>
+        </is>
+      </c>
+      <c r="B12" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A12)</f>
+        <v/>
+      </c>
+      <c r="C12" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A12,Invoices!$F:$F,"Unpaid")</f>
+        <v/>
+      </c>
+      <c r="D12" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$C:$C,A12,Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="E12">
+        <f>COUNTIF(Invoices!$C:$C,A12)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B12" s="4">
-        <f>SUM(B4:B11)</f>
-        <v/>
-      </c>
-      <c r="C12" s="4">
-        <f>SUM(C4:C11)</f>
-        <v/>
-      </c>
-      <c r="D12">
-        <f>SUM(D4:D11)</f>
-        <v/>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="4" t="n"/>
-      <c r="C13" s="4" t="n"/>
+      <c r="B13" s="4">
+        <f>SUM(B4:B12)</f>
+        <v/>
+      </c>
+      <c r="C13" s="4">
+        <f>SUM(C4:C12)</f>
+        <v/>
+      </c>
+      <c r="D13" s="4">
+        <f>SUM(D4:D12)</f>
+        <v/>
+      </c>
+      <c r="E13">
+        <f>SUM(E4:E12)</f>
+        <v/>
+      </c>
     </row>
     <row r="14">
-      <c r="A14" t="inlineStr">
-        <is>
-          <t>Month</t>
-        </is>
-      </c>
-      <c r="B14" s="4" t="inlineStr">
-        <is>
-          <t>Invoiced</t>
-        </is>
-      </c>
+      <c r="B14" s="4" t="n"/>
       <c r="C14" s="4" t="n"/>
+      <c r="D14" s="4" t="n"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-07</t>
-        </is>
-      </c>
-      <c r="B15" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$G$2:$G$61,A15)</f>
-        <v/>
+          <t>Month</t>
+        </is>
+      </c>
+      <c r="B15" s="4" t="inlineStr">
+        <is>
+          <t>Invoiced</t>
+        </is>
       </c>
       <c r="C15" s="4" t="n"/>
+      <c r="D15" s="4" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>2026-08</t>
-        </is>
+      <c r="A16" s="5" t="n">
+        <v>46204</v>
       </c>
       <c r="B16" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$G$2:$G$61,A16)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A16,Invoices!$B:$B,"&lt;"&amp;EDATE(A16,1))</f>
         <v/>
       </c>
       <c r="C16" s="4" t="n"/>
+      <c r="D16" s="4" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>2026-09</t>
-        </is>
+      <c r="A17" s="5" t="n">
+        <v>46235</v>
       </c>
       <c r="B17" s="4">
-        <f>SUMIFS(Invoices!$E$2:$E$61,Invoices!$G$2:$G$61,A17)</f>
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A17,Invoices!$B:$B,"&lt;"&amp;EDATE(A17,1))</f>
         <v/>
       </c>
       <c r="C17" s="4" t="n"/>
+      <c r="D17" s="4" t="n"/>
+    </row>
+    <row r="18">
+      <c r="A18" s="5" t="n">
+        <v>46266</v>
+      </c>
+      <c r="B18" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A18,Invoices!$B:$B,"&lt;"&amp;EDATE(A18,1))</f>
+        <v/>
+      </c>
+      <c r="C18" s="4" t="n"/>
+      <c r="D18" s="4" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="n">
+        <v>46296</v>
+      </c>
+      <c r="B19" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A19,Invoices!$B:$B,"&lt;"&amp;EDATE(A19,1))</f>
+        <v/>
+      </c>
+      <c r="C19" s="4" t="n"/>
+      <c r="D19" s="4" t="n"/>
+    </row>
+    <row r="20">
+      <c r="A20" s="5" t="n">
+        <v>46327</v>
+      </c>
+      <c r="B20" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A20,Invoices!$B:$B,"&lt;"&amp;EDATE(A20,1))</f>
+        <v/>
+      </c>
+      <c r="C20" s="4" t="n"/>
+      <c r="D20" s="4" t="n"/>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="n">
+        <v>46357</v>
+      </c>
+      <c r="B21" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A21,Invoices!$B:$B,"&lt;"&amp;EDATE(A21,1))</f>
+        <v/>
+      </c>
+      <c r="C21" s="4" t="n"/>
+      <c r="D21" s="4" t="n"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="5" t="n">
+        <v>46388</v>
+      </c>
+      <c r="B22" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A22,Invoices!$B:$B,"&lt;"&amp;EDATE(A22,1))</f>
+        <v/>
+      </c>
+      <c r="C22" s="4" t="n"/>
+      <c r="D22" s="4" t="n"/>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="n">
+        <v>46419</v>
+      </c>
+      <c r="B23" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A23,Invoices!$B:$B,"&lt;"&amp;EDATE(A23,1))</f>
+        <v/>
+      </c>
+      <c r="C23" s="4" t="n"/>
+      <c r="D23" s="4" t="n"/>
+    </row>
+    <row r="24">
+      <c r="A24" s="5" t="n">
+        <v>46447</v>
+      </c>
+      <c r="B24" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A24,Invoices!$B:$B,"&lt;"&amp;EDATE(A24,1))</f>
+        <v/>
+      </c>
+      <c r="C24" s="4" t="n"/>
+      <c r="D24" s="4" t="n"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="n">
+        <v>46478</v>
+      </c>
+      <c r="B25" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A25,Invoices!$B:$B,"&lt;"&amp;EDATE(A25,1))</f>
+        <v/>
+      </c>
+      <c r="C25" s="4" t="n"/>
+      <c r="D25" s="4" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="n">
+        <v>46508</v>
+      </c>
+      <c r="B26" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A26,Invoices!$B:$B,"&lt;"&amp;EDATE(A26,1))</f>
+        <v/>
+      </c>
+      <c r="C26" s="4" t="n"/>
+      <c r="D26" s="4" t="n"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="n">
+        <v>46539</v>
+      </c>
+      <c r="B27" s="4">
+        <f>SUMIFS(Invoices!$E:$E,Invoices!$B:$B,"&gt;="&amp;A27,Invoices!$B:$B,"&lt;"&amp;EDATE(A27,1))</f>
+        <v/>
+      </c>
+      <c r="C27" s="4" t="n"/>
+      <c r="D27" s="4" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2768,6 +2695,10 @@
   </sheetPr>
   <dimension ref="A1:E6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
@@ -2802,12 +2733,12 @@
           <t>INV-1030</t>
         </is>
       </c>
-      <c r="B2" s="5" t="n">
+      <c r="B2" s="6" t="n">
         <v>46249</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Oakridge Motors</t>
+          <t>Parkside Dentl</t>
         </is>
       </c>
       <c r="D2" t="n">
@@ -2815,7 +2746,7 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>Same invoice number appears earlier</t>
+          <t>Exact repeat of an earlier row</t>
         </is>
       </c>
     </row>
@@ -2825,7 +2756,7 @@
           <t>INV-1058</t>
         </is>
       </c>
-      <c r="B3" s="5" t="n">
+      <c r="B3" s="6" t="n">
         <v>46219</v>
       </c>
       <c r="C3" t="inlineStr">
@@ -2838,7 +2769,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Same invoice number appears earlier</t>
+          <t>Exact repeat of an earlier row</t>
         </is>
       </c>
     </row>
@@ -2848,7 +2779,7 @@
           <t>INV-1043</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
+      <c r="B4" s="6" t="n">
         <v>46235</v>
       </c>
       <c r="C4" t="inlineStr">
@@ -2861,7 +2792,7 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Same invoice number appears earlier</t>
+          <t>Exact repeat of an earlier row</t>
         </is>
       </c>
     </row>
@@ -2871,7 +2802,7 @@
           <t>INV-1018</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
+      <c r="B5" s="6" t="n">
         <v>46277</v>
       </c>
       <c r="C5" t="inlineStr">
@@ -2884,7 +2815,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Same invoice number appears earlier</t>
+          <t>Exact repeat of an earlier row</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2825,7 @@
           <t>INV-1049</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
+      <c r="B6" s="6" t="n">
         <v>46236</v>
       </c>
       <c r="C6" t="inlineStr">
@@ -2907,7 +2838,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Same invoice number appears earlier</t>
+          <t>Exact repeat of an earlier row</t>
         </is>
       </c>
     </row>
@@ -2922,63 +2853,137 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D4"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="100" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
-          <t>Check</t>
+          <t>Invoice</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>Expected</t>
+          <t>Date</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>Actual</t>
+          <t>Customer</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>OK?</t>
+          <t>Amount</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>Issue</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rows kept = raw rows - blanks - duplicates</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>60</v>
-      </c>
-      <c r="C2">
-        <f>ROWS(Invoices!A2:A61)</f>
-        <v/>
-      </c>
-      <c r="D2">
-        <f>IF(B2=C2,"OK","CHECK")</f>
-        <v/>
+          <t>INV-1012</t>
+        </is>
+      </c>
+      <c r="B2" s="6" t="n">
+        <v>46274</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Riverbend Vets</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>999</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>Same invoice number as a kept row with $640.50: is this a corrected re-issue? Not counted in totals until you decide.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr"/>
+      <c r="B3" t="inlineStr"/>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Parkside Dental / Parkside Dentl</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Names look like a typo of each other: not merged. Fix the spelling on Invoices if they're the same customer.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="64" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="15" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Check</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>Expected</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>Actual</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>OK?</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>LIVE (stay valid as you add rows)</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Customer totals add up to invoice total</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>80632.5</v>
-      </c>
-      <c r="C3">
-        <f>Summary!B12</f>
+          <t>Summary by customer covers every invoice</t>
+        </is>
+      </c>
+      <c r="B3" s="4">
+        <f>SUM(Invoices!$E:$E)</f>
+        <v/>
+      </c>
+      <c r="C3" s="4">
+        <f>Summary!B13</f>
         <v/>
       </c>
       <c r="D3">
@@ -2989,18 +2994,99 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Every status is Paid or Unpaid</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
+          <t>Summary by month covers every invoice</t>
+        </is>
+      </c>
+      <c r="B4" s="4">
+        <f>SUM(Invoices!$E:$E)</f>
+        <v/>
+      </c>
+      <c r="C4" s="4">
+        <f>SUM(Summary!B16:B27)</f>
+        <v/>
+      </c>
+      <c r="D4">
+        <f>IF(ABS(B4-C4)&lt;0.005,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Every status is Paid, Unpaid or Unknown</t>
+        </is>
+      </c>
+      <c r="B5">
+        <f>COUNTA(Invoices!$A:$A)-1</f>
+        <v/>
+      </c>
+      <c r="C5">
+        <f>COUNTIF(Invoices!$F:$F,"Paid")+COUNTIF(Invoices!$F:$F,"Unpaid")+COUNTIF(Invoices!$F:$F,"Unknown")</f>
+        <v/>
+      </c>
+      <c r="D5">
+        <f>IF(ABS(B5-C5)&lt;0.005,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>No invoice number appears twice</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
         <v>0</v>
       </c>
-      <c r="C4">
-        <f>ROWS(Invoices!F2:F61)-COUNTIF(Invoices!F2:F61,"Paid")-COUNTIF(Invoices!F2:F61,"Unpaid")</f>
-        <v/>
-      </c>
-      <c r="D4">
-        <f>IF(B4=C4,"OK","CHECK")</f>
+      <c r="C6">
+        <f>SUMPRODUCT((Invoices!$A$2:$A$561&lt;&gt;"")*(COUNTIF(Invoices!$A$2:$A$561,Invoices!$A$2:$A$561)&gt;1))</f>
+        <v/>
+      </c>
+      <c r="D6">
+        <f>IF(ABS(B6-C6)&lt;0.005,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>CLEAN-UP RECONCILIATION (vs the original export, as delivered; adding new rows will change these)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Rows: original export = kept + duplicates + needs review + blank</t>
+        </is>
+      </c>
+      <c r="B8" s="7" t="n">
+        <v>67</v>
+      </c>
+      <c r="C8" s="7">
+        <f>(COUNTA(Invoices!$A:$A)-1)+(COUNTA('Duplicates removed'!$A:$A)-1)+COUNTIF('Needs review'!$E:$E,"Same invoice*")+1</f>
+        <v/>
+      </c>
+      <c r="D8">
+        <f>IF(ABS(B8-C8)&lt;0.005,"OK","CHECK")</f>
+        <v/>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Money: original export total = kept + duplicates + needs review</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>88063.5</v>
+      </c>
+      <c r="C9" s="4">
+        <f>SUM(Invoices!$E:$E)+SUM('Duplicates removed'!$D:$D)+SUM('Needs review'!$D:$D)</f>
+        <v/>
+      </c>
+      <c r="D9">
+        <f>IF(ABS(B9-C9)&lt;0.005,"OK","CHECK")</f>
         <v/>
       </c>
     </row>

</xml_diff>